<commit_message>
cambios excel y docx
</commit_message>
<xml_diff>
--- a/Docs/TablasDatos-Lab6.xlsx
+++ b/Docs/TablasDatos-Lab6.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="21" documentId="13_ncr:1_{FD33DA02-4501-4B58-9D83-E0FFBD1B4D85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1E9FD380-61A2-49FF-B83F-A65988C44B82}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="767" xr2:uid="{D82936D8-D2C9-4EB2-9CBC-3665F65B95FD}"/>
+    <workbookView xWindow="1300" yWindow="3110" windowWidth="14400" windowHeight="8170" tabRatio="767" xr2:uid="{D82936D8-D2C9-4EB2-9CBC-3665F65B95FD}"/>
   </bookViews>
   <sheets>
     <sheet name="Datos Lab6" sheetId="1" r:id="rId1"/>
@@ -2903,7 +2903,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
     <xdr:pos x="0" y="0"/>
-    <xdr:ext cx="9297051" cy="6073205"/>
+    <xdr:ext cx="9293175" cy="6067778"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart 1">
@@ -2936,7 +2936,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
     <xdr:pos x="0" y="0"/>
-    <xdr:ext cx="9297051" cy="6073205"/>
+    <xdr:ext cx="9293175" cy="6067778"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart 1">
@@ -3444,6 +3444,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010023858CF01A2EF24688B692775F4C60A4" ma:contentTypeVersion="17" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="af74a0f8eb440a60883e9dd833f0742f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="164883f8-7691-4ecf-b54a-664c0d0edefe" xmlns:ns3="85e30bcc-d76c-4413-8e4d-2dce22fb0743" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f5ceeff32ffca1089660572a8ebd1782" ns2:_="" ns3:_="">
     <xsd:import namespace="164883f8-7691-4ecf-b54a-664c0d0edefe"/>
@@ -3692,15 +3701,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97C5E1E0-C817-4769-9D2D-1DC296B681FA}">
   <ds:schemaRefs>
@@ -3713,6 +3713,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F8DF3742-38F2-4B99-B335-CC4F04ED9F45}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E10B9E65-6C88-4633-81F7-F02338B2B10B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3729,12 +3737,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F8DF3742-38F2-4B99-B335-CC4F04ED9F45}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>